<commit_message>
Configure static ngrok domain, update backend URL, and add feed server enhancements
</commit_message>
<xml_diff>
--- a/ppe_log.xlsx
+++ b/ppe_log.xlsx
@@ -413,8 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:H9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
@@ -471,11 +471,16 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-07-14 17:04:47</t>
+          <t>2026-09-05 07:35:25</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>VIOLATION</t>
+        </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -489,26 +494,21 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>screenshots\track_3_1784028887965.jpg</t>
+          <t>screenshots/track_4_1788573925559.jpg</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-07-14 17:05:19</t>
+          <t>2026-09-05 07:36:20</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
           <t>VIOLATION</t>
         </is>
       </c>
@@ -519,18 +519,18 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>screenshots\track_19_1784028919726.jpg</t>
+          <t>screenshots/track_12_1788573980046.jpg</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-14 17:05:42</t>
+          <t>2026-09-05 07:42:03</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -544,20 +544,20 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>screenshots\track_54_1784028942298.jpg</t>
+          <t>screenshots/track_29_1788574323598.jpg</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-07-14 17:05:50</t>
+          <t>2026-09-05 07:47:56</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>92</v>
-      </c>
-      <c r="D5" t="inlineStr">
+        <v>41</v>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>VIOLATION</t>
         </is>
@@ -569,51 +569,46 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>screenshots\track_92_1784028950887.jpg</t>
+          <t>screenshots/track_41_1788574676738.jpg</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-07-14 17:12:40</t>
+          <t>2026-09-05 07:48:37</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2</v>
+        <v>58</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>OK</t>
+          <t>VIOLATION</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Compliant</t>
+          <t>Non-Compliant</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>screenshots\track_2_1784029360139.jpg</t>
+          <t>screenshots/track_58_1788574717587.jpg</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-07-14 17:13:05</t>
+          <t>2026-09-05 08:39:54</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>17</v>
+        <v>131</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
           <t>VIOLATION</t>
         </is>
       </c>
@@ -624,20 +619,20 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>screenshots\track_17_1784029385041.jpg</t>
+          <t>screenshots/track_131_1788577794979.jpg</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-07-14 17:13:25</t>
+          <t>2026-09-05 09:14:11</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>23</v>
-      </c>
-      <c r="D8" t="inlineStr">
+        <v>166</v>
+      </c>
+      <c r="E8" t="inlineStr">
         <is>
           <t>VIOLATION</t>
         </is>
@@ -649,24 +644,27 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>screenshots\track_23_1784029405674.jpg</t>
+          <t>screenshots/track_166_1788579851432.jpg</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-07-14 17:13:30</t>
+          <t>2026-09-05 09:53:19</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>29</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>VIOLATION</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>Non-Compliant</t>
@@ -674,192 +672,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>screenshots\track_29_1784029410737.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>2026-07-14 17:13:40</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>72</v>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Non-Compliant</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>screenshots\track_72_1784029420861.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>2026-07-14 17:13:52</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>84</v>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>Non-Compliant</t>
-        </is>
-      </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>screenshots\track_84_1784029432201.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>2026-07-14 17:13:57</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>100</v>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Non-Compliant</t>
-        </is>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>screenshots\track_100_1784029437204.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>2026-07-14 17:14:02</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>144</v>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Non-Compliant</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>screenshots\track_144_1784029442381.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>2026-07-14 17:14:08</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>163</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>Non-Compliant</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>screenshots\track_163_1784029448254.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2026-07-14 17:14:14</t>
-        </is>
-      </c>
-      <c r="B15" t="n">
-        <v>199</v>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Non-Compliant</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>screenshots\track_199_1784029454131.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-08-01 17:26:43</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>4</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>VIOLATION</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>Non-Compliant</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>screenshots/track_4_1785585403579.jpg</t>
+          <t>screenshots/track_4_1788582199190.jpg</t>
         </is>
       </c>
     </row>

</xml_diff>